<commit_message>
Import: keep the two years before the export date instead of a fixed cutoff
The parser ignored everything before 2025-02-01 (when one user's Watch data
started), so older exports imported nothing and longer histories lost years.
The window now ends at the export's <ExportDate> (today if missing) and
reaches back 2 years; a fixed cutoff can still be passed explicitly.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Cases'!$A$1:$G$234</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Cases'!$A$1:$G$236</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G234"/>
+  <dimension ref="A1:G236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="G2" s="5" t="n">
-        <v>8.699999999999999</v>
+        <v>11.3</v>
       </c>
     </row>
     <row r="3">
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="G3" s="5" t="n">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="4">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="G4" s="5" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="5">
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="G5" s="5" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="6">
@@ -851,7 +851,7 @@
         </is>
       </c>
       <c r="G10" s="5" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="11">
@@ -884,7 +884,7 @@
         </is>
       </c>
       <c r="G11" s="5" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="12">
@@ -917,7 +917,7 @@
         </is>
       </c>
       <c r="G12" s="5" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="13">
@@ -983,7 +983,7 @@
         </is>
       </c>
       <c r="G14" s="5" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="15">
@@ -1016,7 +1016,7 @@
         </is>
       </c>
       <c r="G15" s="5" t="n">
-        <v>1.9</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="16">
@@ -1049,7 +1049,7 @@
         </is>
       </c>
       <c r="G16" s="5" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="G17" s="5" t="n">
-        <v>0.9</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="18">
@@ -1115,7 +1115,7 @@
         </is>
       </c>
       <c r="G18" s="5" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="19">
@@ -1148,7 +1148,7 @@
         </is>
       </c>
       <c r="G19" s="5" t="n">
-        <v>2</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="20">
@@ -1181,7 +1181,7 @@
         </is>
       </c>
       <c r="G20" s="5" t="n">
-        <v>2.3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="G21" s="5" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -1247,7 +1247,7 @@
         </is>
       </c>
       <c r="G22" s="5" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="23">
@@ -1346,7 +1346,7 @@
         </is>
       </c>
       <c r="G25" s="5" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="26">
@@ -1379,7 +1379,7 @@
         </is>
       </c>
       <c r="G26" s="5" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="27">
@@ -1412,7 +1412,7 @@
         </is>
       </c>
       <c r="G27" s="5" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="28">
@@ -1511,7 +1511,7 @@
         </is>
       </c>
       <c r="G30" s="5" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="31">
@@ -1544,7 +1544,7 @@
         </is>
       </c>
       <c r="G31" s="5" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="32">
@@ -1577,7 +1577,7 @@
         </is>
       </c>
       <c r="G32" s="5" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="33">
@@ -1742,7 +1742,7 @@
         </is>
       </c>
       <c r="G37" s="5" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="38">
@@ -1841,7 +1841,7 @@
         </is>
       </c>
       <c r="G40" s="5" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="41">
@@ -1907,7 +1907,7 @@
         </is>
       </c>
       <c r="G42" s="5" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="43">
@@ -1940,7 +1940,7 @@
         </is>
       </c>
       <c r="G43" s="5" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="44">
@@ -1973,7 +1973,7 @@
         </is>
       </c>
       <c r="G44" s="5" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="45">
@@ -2006,7 +2006,7 @@
         </is>
       </c>
       <c r="G45" s="5" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="46">
@@ -2072,7 +2072,7 @@
         </is>
       </c>
       <c r="G47" s="5" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="48">
@@ -2171,7 +2171,7 @@
         </is>
       </c>
       <c r="G50" s="5" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="51">
@@ -2402,7 +2402,7 @@
         </is>
       </c>
       <c r="G57" s="5" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="58">
@@ -2567,7 +2567,7 @@
         </is>
       </c>
       <c r="G62" s="5" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="63">
@@ -2600,7 +2600,7 @@
         </is>
       </c>
       <c r="G63" s="5" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="64">
@@ -3425,7 +3425,7 @@
         </is>
       </c>
       <c r="G88" s="5" t="n">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="89">
@@ -3458,7 +3458,7 @@
         </is>
       </c>
       <c r="G89" s="5" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="90">
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="G91" s="5" t="n">
-        <v>1.8</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="92">
@@ -3689,7 +3689,7 @@
         </is>
       </c>
       <c r="G96" s="5" t="n">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="97">
@@ -3722,7 +3722,7 @@
         </is>
       </c>
       <c r="G97" s="5" t="n">
-        <v>1.2</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="98">
@@ -3755,7 +3755,7 @@
         </is>
       </c>
       <c r="G98" s="5" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="99">
@@ -4019,7 +4019,7 @@
         </is>
       </c>
       <c r="G106" s="5" t="n">
-        <v>11.5</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="107">
@@ -4052,7 +4052,7 @@
         </is>
       </c>
       <c r="G107" s="5" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="108">
@@ -4085,7 +4085,7 @@
         </is>
       </c>
       <c r="G108" s="5" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="109">
@@ -4151,7 +4151,7 @@
         </is>
       </c>
       <c r="G110" s="5" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="111">
@@ -4217,7 +4217,7 @@
         </is>
       </c>
       <c r="G112" s="5" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="113">
@@ -4250,7 +4250,7 @@
         </is>
       </c>
       <c r="G113" s="5" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="114">
@@ -4316,7 +4316,7 @@
         </is>
       </c>
       <c r="G115" s="5" t="n">
-        <v>4.4</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="116">
@@ -4349,7 +4349,7 @@
         </is>
       </c>
       <c r="G116" s="5" t="n">
-        <v>16.5</v>
+        <v>24.5</v>
       </c>
     </row>
     <row r="117">
@@ -4382,7 +4382,7 @@
         </is>
       </c>
       <c r="G117" s="5" t="n">
-        <v>219.1</v>
+        <v>232.3</v>
       </c>
     </row>
     <row r="118">
@@ -4415,7 +4415,7 @@
         </is>
       </c>
       <c r="G118" s="5" t="n">
-        <v>16.5</v>
+        <v>15.6</v>
       </c>
     </row>
     <row r="119">
@@ -4448,7 +4448,7 @@
         </is>
       </c>
       <c r="G119" s="5" t="n">
-        <v>13</v>
+        <v>14.7</v>
       </c>
     </row>
     <row r="120">
@@ -4481,7 +4481,7 @@
         </is>
       </c>
       <c r="G120" s="5" t="n">
-        <v>1</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="121">
@@ -4514,7 +4514,7 @@
         </is>
       </c>
       <c r="G121" s="5" t="n">
-        <v>14.2</v>
+        <v>28.4</v>
       </c>
     </row>
     <row r="122">
@@ -4547,7 +4547,7 @@
         </is>
       </c>
       <c r="G122" s="5" t="n">
-        <v>16.1</v>
+        <v>15.6</v>
       </c>
     </row>
     <row r="123">
@@ -4580,7 +4580,7 @@
         </is>
       </c>
       <c r="G123" s="5" t="n">
-        <v>6.2</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="124">
@@ -4613,7 +4613,7 @@
         </is>
       </c>
       <c r="G124" s="5" t="n">
-        <v>1.8</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="125">
@@ -4646,7 +4646,7 @@
         </is>
       </c>
       <c r="G125" s="5" t="n">
-        <v>1.4</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="126">
@@ -4679,7 +4679,7 @@
         </is>
       </c>
       <c r="G126" s="5" t="n">
-        <v>0.7</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="127">
@@ -4712,7 +4712,7 @@
         </is>
       </c>
       <c r="G127" s="5" t="n">
-        <v>0.9</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="128">
@@ -4745,7 +4745,7 @@
         </is>
       </c>
       <c r="G128" s="5" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="129">
@@ -4769,7 +4769,7 @@
       </c>
       <c r="E129" s="3" t="inlineStr">
         <is>
-          <t>ignores records before the cutoff and lines it does not know (header, DTD)</t>
+          <t>keeps the two years before the export date and ignores lines it does not know (header, DTD)</t>
         </is>
       </c>
       <c r="F129" s="4" t="inlineStr">
@@ -4778,7 +4778,7 @@
         </is>
       </c>
       <c r="G129" s="5" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="130">
@@ -4802,7 +4802,7 @@
       </c>
       <c r="E130" s="3" t="inlineStr">
         <is>
-          <t>fails clearly when the export has no usable records</t>
+          <t>measures the window from the export date, so an old export still imports</t>
         </is>
       </c>
       <c r="F130" s="4" t="inlineStr">
@@ -4811,7 +4811,7 @@
         </is>
       </c>
       <c r="G130" s="5" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="131">
@@ -4830,12 +4830,12 @@
       </c>
       <c r="D131" s="3" t="inlineStr">
         <is>
-          <t>createLineSplitter</t>
+          <t>createParser</t>
         </is>
       </c>
       <c r="E131" s="3" t="inlineStr">
         <is>
-          <t>rebuilds lines split across chunks, including CRLF endings</t>
+          <t>falls back to two years before today without an export date, and a fixed cutoff overrides both</t>
         </is>
       </c>
       <c r="F131" s="4" t="inlineStr">
@@ -4844,7 +4844,7 @@
         </is>
       </c>
       <c r="G131" s="5" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="132">
@@ -4853,22 +4853,22 @@
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>storage</t>
+          <t>parse-core</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>src/health/storage.test.ts</t>
+          <t>src/health/import/parse-core.test.ts</t>
         </is>
       </c>
       <c r="D132" s="3" t="inlineStr">
         <is>
-          <t>health snapshot encoding</t>
+          <t>createParser</t>
         </is>
       </c>
       <c r="E132" s="3" t="inlineStr">
         <is>
-          <t>round-trips a dataset through the compressed form</t>
+          <t>fails clearly when the export has no usable records</t>
         </is>
       </c>
       <c r="F132" s="4" t="inlineStr">
@@ -4877,7 +4877,7 @@
         </is>
       </c>
       <c r="G132" s="5" t="n">
-        <v>7</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="133">
@@ -4886,22 +4886,22 @@
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>storage</t>
+          <t>parse-core</t>
         </is>
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>src/health/storage.test.ts</t>
+          <t>src/health/import/parse-core.test.ts</t>
         </is>
       </c>
       <c r="D133" s="3" t="inlineStr">
         <is>
-          <t>health snapshot encoding</t>
+          <t>createLineSplitter</t>
         </is>
       </c>
       <c r="E133" s="3" t="inlineStr">
         <is>
-          <t>treats damaged or foreign snapshots as no data instead of crashing</t>
+          <t>rebuilds lines split across chunks, including CRLF endings</t>
         </is>
       </c>
       <c r="F133" s="4" t="inlineStr">
@@ -4910,7 +4910,7 @@
         </is>
       </c>
       <c r="G133" s="5" t="n">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="134">
@@ -4929,12 +4929,12 @@
       </c>
       <c r="D134" s="3" t="inlineStr">
         <is>
-          <t>isHealthData</t>
+          <t>health snapshot encoding</t>
         </is>
       </c>
       <c r="E134" s="3" t="inlineStr">
         <is>
-          <t>accepts a well-formed dataset</t>
+          <t>round-trips a dataset through the compressed form</t>
         </is>
       </c>
       <c r="F134" s="4" t="inlineStr">
@@ -4943,7 +4943,7 @@
         </is>
       </c>
       <c r="G134" s="5" t="n">
-        <v>0.6</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="135">
@@ -4962,12 +4962,12 @@
       </c>
       <c r="D135" s="3" t="inlineStr">
         <is>
-          <t>isHealthData</t>
+          <t>health snapshot encoding</t>
         </is>
       </c>
       <c r="E135" s="3" t="inlineStr">
         <is>
-          <t>rejects a bad date key</t>
+          <t>treats damaged or foreign snapshots as no data instead of crashing</t>
         </is>
       </c>
       <c r="F135" s="4" t="inlineStr">
@@ -4976,7 +4976,7 @@
         </is>
       </c>
       <c r="G135" s="5" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="136">
@@ -5000,7 +5000,7 @@
       </c>
       <c r="E136" s="3" t="inlineStr">
         <is>
-          <t>rejects firstDay after lastDay</t>
+          <t>accepts a well-formed dataset</t>
         </is>
       </c>
       <c r="F136" s="4" t="inlineStr">
@@ -5033,7 +5033,7 @@
       </c>
       <c r="E137" s="3" t="inlineStr">
         <is>
-          <t>rejects a day missing its parts</t>
+          <t>rejects a bad date key</t>
         </is>
       </c>
       <c r="F137" s="4" t="inlineStr">
@@ -5042,7 +5042,7 @@
         </is>
       </c>
       <c r="G137" s="5" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="138">
@@ -5066,7 +5066,7 @@
       </c>
       <c r="E138" s="3" t="inlineStr">
         <is>
-          <t>rejects workouts that are not workouts</t>
+          <t>rejects firstDay after lastDay</t>
         </is>
       </c>
       <c r="F138" s="4" t="inlineStr">
@@ -5075,7 +5075,7 @@
         </is>
       </c>
       <c r="G138" s="5" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="139">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="E139" s="3" t="inlineStr">
         <is>
-          <t>rejects a missing profile</t>
+          <t>rejects a day missing its parts</t>
         </is>
       </c>
       <c r="F139" s="4" t="inlineStr">
@@ -5108,7 +5108,7 @@
         </is>
       </c>
       <c r="G139" s="5" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="140">
@@ -5127,12 +5127,12 @@
       </c>
       <c r="D140" s="3" t="inlineStr">
         <is>
-          <t>saving on the device</t>
+          <t>isHealthData</t>
         </is>
       </c>
       <c r="E140" s="3" t="inlineStr">
         <is>
-          <t>saves and loads back the snapshot</t>
+          <t>rejects workouts that are not workouts</t>
         </is>
       </c>
       <c r="F140" s="4" t="inlineStr">
@@ -5141,7 +5141,7 @@
         </is>
       </c>
       <c r="G140" s="5" t="n">
-        <v>2.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="141">
@@ -5160,12 +5160,12 @@
       </c>
       <c r="D141" s="3" t="inlineStr">
         <is>
-          <t>saving on the device</t>
+          <t>isHealthData</t>
         </is>
       </c>
       <c r="E141" s="3" t="inlineStr">
         <is>
-          <t>explains when the browser cannot store anything (e.g. Private Browsing)</t>
+          <t>rejects a missing profile</t>
         </is>
       </c>
       <c r="F141" s="4" t="inlineStr">
@@ -5174,7 +5174,7 @@
         </is>
       </c>
       <c r="G141" s="5" t="n">
-        <v>1.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="142">
@@ -5198,7 +5198,7 @@
       </c>
       <c r="E142" s="3" t="inlineStr">
         <is>
-          <t>explains when the device is out of space</t>
+          <t>saves and loads back the snapshot</t>
         </is>
       </c>
       <c r="F142" s="4" t="inlineStr">
@@ -5207,7 +5207,7 @@
         </is>
       </c>
       <c r="G142" s="5" t="n">
-        <v>0.9</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="143">
@@ -5231,7 +5231,7 @@
       </c>
       <c r="E143" s="3" t="inlineStr">
         <is>
-          <t>Delete all data removes every bodyn key and leaves other sites’ keys alone</t>
+          <t>explains when the browser cannot store anything (e.g. Private Browsing)</t>
         </is>
       </c>
       <c r="F143" s="4" t="inlineStr">
@@ -5240,7 +5240,7 @@
         </is>
       </c>
       <c r="G143" s="5" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="144">
@@ -5259,12 +5259,12 @@
       </c>
       <c r="D144" s="3" t="inlineStr">
         <is>
-          <t>createStoredProvider</t>
+          <t>saving on the device</t>
         </is>
       </c>
       <c r="E144" s="3" t="inlineStr">
         <is>
-          <t>serves days, gap-filled ranges, workouts by date and recent HR samples</t>
+          <t>explains when the device is out of space</t>
         </is>
       </c>
       <c r="F144" s="4" t="inlineStr">
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="G144" s="5" t="n">
-        <v>1.6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="145">
@@ -5292,12 +5292,12 @@
       </c>
       <c r="D145" s="3" t="inlineStr">
         <is>
-          <t>createStoredProvider</t>
+          <t>saving on the device</t>
         </is>
       </c>
       <c r="E145" s="3" t="inlineStr">
         <is>
-          <t>is empty but safe to call before anything is imported</t>
+          <t>Delete all data removes every bodyn key and leaves other sites’ keys alone</t>
         </is>
       </c>
       <c r="F145" s="4" t="inlineStr">
@@ -5306,7 +5306,7 @@
         </is>
       </c>
       <c r="G145" s="5" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="146">
@@ -5315,22 +5315,22 @@
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>Units</t>
+          <t>storage</t>
         </is>
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>src/lib/units.test.ts</t>
+          <t>src/health/storage.test.ts</t>
         </is>
       </c>
       <c r="D146" s="3" t="inlineStr">
         <is>
-          <t>unit conversion</t>
+          <t>createStoredProvider</t>
         </is>
       </c>
       <c r="E146" s="3" t="inlineStr">
         <is>
-          <t>distance: km passes through, mi converts</t>
+          <t>serves days, gap-filled ranges, workouts by date and recent HR samples</t>
         </is>
       </c>
       <c r="F146" s="4" t="inlineStr">
@@ -5339,7 +5339,7 @@
         </is>
       </c>
       <c r="G146" s="5" t="n">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="147">
@@ -5348,22 +5348,22 @@
       </c>
       <c r="B147" s="2" t="inlineStr">
         <is>
-          <t>Units</t>
+          <t>storage</t>
         </is>
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>src/lib/units.test.ts</t>
+          <t>src/health/storage.test.ts</t>
         </is>
       </c>
       <c r="D147" s="3" t="inlineStr">
         <is>
-          <t>unit conversion</t>
+          <t>createStoredProvider</t>
         </is>
       </c>
       <c r="E147" s="3" t="inlineStr">
         <is>
-          <t>weight: kg passes through, lb converts</t>
+          <t>is empty but safe to call before anything is imported</t>
         </is>
       </c>
       <c r="F147" s="4" t="inlineStr">
@@ -5396,7 +5396,7 @@
       </c>
       <c r="E148" s="3" t="inlineStr">
         <is>
-          <t>energy: kcal passes through, kJ converts</t>
+          <t>distance: km passes through, mi converts</t>
         </is>
       </c>
       <c r="F148" s="4" t="inlineStr">
@@ -5405,7 +5405,7 @@
         </is>
       </c>
       <c r="G148" s="5" t="n">
-        <v>0.3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="149">
@@ -5429,7 +5429,7 @@
       </c>
       <c r="E149" s="3" t="inlineStr">
         <is>
-          <t>labels match the unit</t>
+          <t>weight: kg passes through, lb converts</t>
         </is>
       </c>
       <c r="F149" s="4" t="inlineStr">
@@ -5438,7 +5438,7 @@
         </is>
       </c>
       <c r="G149" s="5" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="150">
@@ -5447,22 +5447,22 @@
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>Metrics engine</t>
+          <t>Units</t>
         </is>
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>src/metrics/engine.test.ts</t>
+          <t>src/lib/units.test.ts</t>
         </is>
       </c>
       <c r="D150" s="3" t="inlineStr">
         <is>
-          <t>math helpers</t>
+          <t>unit conversion</t>
         </is>
       </c>
       <c r="E150" s="3" t="inlineStr">
         <is>
-          <t>normCdf is a proper CDF</t>
+          <t>energy: kcal passes through, kJ converts</t>
         </is>
       </c>
       <c r="F150" s="4" t="inlineStr">
@@ -5471,7 +5471,7 @@
         </is>
       </c>
       <c r="G150" s="5" t="n">
-        <v>2.4</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="151">
@@ -5480,22 +5480,22 @@
       </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
-          <t>Metrics engine</t>
+          <t>Units</t>
         </is>
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>src/metrics/engine.test.ts</t>
+          <t>src/lib/units.test.ts</t>
         </is>
       </c>
       <c r="D151" s="3" t="inlineStr">
         <is>
-          <t>math helpers</t>
+          <t>unit conversion</t>
         </is>
       </c>
       <c r="E151" s="3" t="inlineStr">
         <is>
-          <t>bands and labels</t>
+          <t>labels match the unit</t>
         </is>
       </c>
       <c r="F151" s="4" t="inlineStr">
@@ -5504,7 +5504,7 @@
         </is>
       </c>
       <c r="G151" s="5" t="n">
-        <v>0.7</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="152">
@@ -5528,7 +5528,7 @@
       </c>
       <c r="E152" s="3" t="inlineStr">
         <is>
-          <t>toStrain is 0 at 0, log-shaped and capped at 21</t>
+          <t>normCdf is a proper CDF</t>
         </is>
       </c>
       <c r="F152" s="4" t="inlineStr">
@@ -5537,7 +5537,7 @@
         </is>
       </c>
       <c r="G152" s="5" t="n">
-        <v>0.3</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="153">
@@ -5561,7 +5561,7 @@
       </c>
       <c r="E153" s="3" t="inlineStr">
         <is>
-          <t>zoneMinutes buckets by % of max HR</t>
+          <t>bands and labels</t>
         </is>
       </c>
       <c r="F153" s="4" t="inlineStr">
@@ -5570,7 +5570,7 @@
         </is>
       </c>
       <c r="G153" s="5" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="154">
@@ -5589,12 +5589,12 @@
       </c>
       <c r="D154" s="3" t="inlineStr">
         <is>
-          <t>sleep score</t>
+          <t>math helpers</t>
         </is>
       </c>
       <c r="E154" s="3" t="inlineStr">
         <is>
-          <t>is high for a full, efficient, restorative night and lower when short</t>
+          <t>toStrain is 0 at 0, log-shaped and capped at 21</t>
         </is>
       </c>
       <c r="F154" s="4" t="inlineStr">
@@ -5603,7 +5603,7 @@
         </is>
       </c>
       <c r="G154" s="5" t="n">
-        <v>3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="155">
@@ -5622,12 +5622,12 @@
       </c>
       <c r="D155" s="3" t="inlineStr">
         <is>
-          <t>sleep score</t>
+          <t>math helpers</t>
         </is>
       </c>
       <c r="E155" s="3" t="inlineStr">
         <is>
-          <t>sleep need rises after a high-strain day</t>
+          <t>zoneMinutes buckets by % of max HR</t>
         </is>
       </c>
       <c r="F155" s="4" t="inlineStr">
@@ -5636,7 +5636,7 @@
         </is>
       </c>
       <c r="G155" s="5" t="n">
-        <v>1.5</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="156">
@@ -5660,7 +5660,7 @@
       </c>
       <c r="E156" s="3" t="inlineStr">
         <is>
-          <t>is null without a sleep session</t>
+          <t>is high for a full, efficient, restorative night and lower when short</t>
         </is>
       </c>
       <c r="F156" s="4" t="inlineStr">
@@ -5669,7 +5669,7 @@
         </is>
       </c>
       <c r="G156" s="5" t="n">
-        <v>0.3</v>
+        <v>3</v>
       </c>
     </row>
     <row r="157">
@@ -5688,12 +5688,12 @@
       </c>
       <c r="D157" s="3" t="inlineStr">
         <is>
-          <t>recovery</t>
+          <t>sleep score</t>
         </is>
       </c>
       <c r="E157" s="3" t="inlineStr">
         <is>
-          <t>rises with higher HRV / lower RHR and falls with the opposite, vs. own baseline</t>
+          <t>sleep need rises after a high-strain day</t>
         </is>
       </c>
       <c r="F157" s="4" t="inlineStr">
@@ -5702,7 +5702,7 @@
         </is>
       </c>
       <c r="G157" s="5" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="158">
@@ -5721,12 +5721,12 @@
       </c>
       <c r="D158" s="3" t="inlineStr">
         <is>
-          <t>recovery</t>
+          <t>sleep score</t>
         </is>
       </c>
       <c r="E158" s="3" t="inlineStr">
         <is>
-          <t>an average day sits near the middle</t>
+          <t>is null without a sleep session</t>
         </is>
       </c>
       <c r="F158" s="4" t="inlineStr">
@@ -5735,7 +5735,7 @@
         </is>
       </c>
       <c r="G158" s="5" t="n">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="159">
@@ -5759,7 +5759,7 @@
       </c>
       <c r="E159" s="3" t="inlineStr">
         <is>
-          <t>needs a baseline before it scores</t>
+          <t>rises with higher HRV / lower RHR and falls with the opposite, vs. own baseline</t>
         </is>
       </c>
       <c r="F159" s="4" t="inlineStr">
@@ -5768,7 +5768,7 @@
         </is>
       </c>
       <c r="G159" s="5" t="n">
-        <v>0.3</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="160">
@@ -5787,12 +5787,12 @@
       </c>
       <c r="D160" s="3" t="inlineStr">
         <is>
-          <t>strain</t>
+          <t>recovery</t>
         </is>
       </c>
       <c r="E160" s="3" t="inlineStr">
         <is>
-          <t>is null with no heart-rate data and ~0 for a resting day</t>
+          <t>an average day sits near the middle</t>
         </is>
       </c>
       <c r="F160" s="4" t="inlineStr">
@@ -5801,7 +5801,7 @@
         </is>
       </c>
       <c r="G160" s="5" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="161">
@@ -5820,12 +5820,12 @@
       </c>
       <c r="D161" s="3" t="inlineStr">
         <is>
-          <t>strain</t>
+          <t>recovery</t>
         </is>
       </c>
       <c r="E161" s="3" t="inlineStr">
         <is>
-          <t>increases with time at high heart rate and stays within 0–21</t>
+          <t>needs a baseline before it scores</t>
         </is>
       </c>
       <c r="F161" s="4" t="inlineStr">
@@ -5834,7 +5834,7 @@
         </is>
       </c>
       <c r="G161" s="5" t="n">
-        <v>1.3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="162">
@@ -5853,12 +5853,12 @@
       </c>
       <c r="D162" s="3" t="inlineStr">
         <is>
-          <t>health-prefs overrides</t>
+          <t>strain</t>
         </is>
       </c>
       <c r="E162" s="3" t="inlineStr">
         <is>
-          <t>a manual sleep goal changes needMin, even for an already-computed date (cache invalidation)</t>
+          <t>is null with no heart-rate data and ~0 for a resting day</t>
         </is>
       </c>
       <c r="F162" s="4" t="inlineStr">
@@ -5867,7 +5867,7 @@
         </is>
       </c>
       <c r="G162" s="5" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="163">
@@ -5886,12 +5886,12 @@
       </c>
       <c r="D163" s="3" t="inlineStr">
         <is>
-          <t>health-prefs overrides</t>
+          <t>strain</t>
         </is>
       </c>
       <c r="E163" s="3" t="inlineStr">
         <is>
-          <t>a manual max/resting HR overrides the computed profile and changes strain</t>
+          <t>increases with time at high heart rate and stays within 0–21</t>
         </is>
       </c>
       <c r="F163" s="4" t="inlineStr">
@@ -5900,7 +5900,7 @@
         </is>
       </c>
       <c r="G163" s="5" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="164">
@@ -5924,7 +5924,7 @@
       </c>
       <c r="E164" s="3" t="inlineStr">
         <is>
-          <t>custom zone bands change zone minutes for an already-computed date</t>
+          <t>a manual sleep goal changes needMin, even for an already-computed date (cache invalidation)</t>
         </is>
       </c>
       <c r="F164" s="4" t="inlineStr">
@@ -5933,7 +5933,7 @@
         </is>
       </c>
       <c r="G164" s="5" t="n">
-        <v>0.9</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="165">
@@ -5952,12 +5952,12 @@
       </c>
       <c r="D165" s="3" t="inlineStr">
         <is>
-          <t>HRV outlier rein-in</t>
+          <t>health-prefs overrides</t>
         </is>
       </c>
       <c r="E165" s="3" t="inlineStr">
         <is>
-          <t>one artefact reading cannot run away with the score</t>
+          <t>a manual max/resting HR overrides the computed profile and changes strain</t>
         </is>
       </c>
       <c r="F165" s="4" t="inlineStr">
@@ -5966,7 +5966,7 @@
         </is>
       </c>
       <c r="G165" s="5" t="n">
-        <v>0.5</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="166">
@@ -5985,12 +5985,12 @@
       </c>
       <c r="D166" s="3" t="inlineStr">
         <is>
-          <t>HRV outlier rein-in</t>
+          <t>health-prefs overrides</t>
         </is>
       </c>
       <c r="E166" s="3" t="inlineStr">
         <is>
-          <t>leaves an ordinary night completely alone</t>
+          <t>custom zone bands change zone minutes for an already-computed date</t>
         </is>
       </c>
       <c r="F166" s="4" t="inlineStr">
@@ -5999,7 +5999,7 @@
         </is>
       </c>
       <c r="G166" s="5" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="167">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="E167" s="3" t="inlineStr">
         <is>
-          <t>a genuinely great night still scores well</t>
+          <t>one artefact reading cannot run away with the score</t>
         </is>
       </c>
       <c r="F167" s="4" t="inlineStr">
@@ -6032,7 +6032,7 @@
         </is>
       </c>
       <c r="G167" s="5" t="n">
-        <v>0.4</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="168">
@@ -6056,7 +6056,7 @@
       </c>
       <c r="E168" s="3" t="inlineStr">
         <is>
-          <t>still works for a night with no per-reading detail</t>
+          <t>leaves an ordinary night completely alone</t>
         </is>
       </c>
       <c r="F168" s="4" t="inlineStr">
@@ -6065,7 +6065,7 @@
         </is>
       </c>
       <c r="G168" s="5" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="169">
@@ -6089,7 +6089,7 @@
       </c>
       <c r="E169" s="3" t="inlineStr">
         <is>
-          <t>resting heart rate can be read from your sleep instead of the daily figure</t>
+          <t>a genuinely great night still scores well</t>
         </is>
       </c>
       <c r="F169" s="4" t="inlineStr">
@@ -6098,7 +6098,7 @@
         </is>
       </c>
       <c r="G169" s="5" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="170">
@@ -6107,22 +6107,22 @@
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>Fitness age</t>
+          <t>Metrics engine</t>
         </is>
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>src/metrics/fitness-profile.test.ts</t>
+          <t>src/metrics/engine.test.ts</t>
         </is>
       </c>
       <c r="D170" s="3" t="inlineStr">
         <is>
-          <t>metricProfile</t>
+          <t>HRV outlier rein-in</t>
         </is>
       </c>
       <c r="E170" s="3" t="inlineStr">
         <is>
-          <t>a higher-is-better metric trending up over the last 30 days reads "good"</t>
+          <t>still works for a night with no per-reading detail</t>
         </is>
       </c>
       <c r="F170" s="4" t="inlineStr">
@@ -6131,7 +6131,7 @@
         </is>
       </c>
       <c r="G170" s="5" t="n">
-        <v>3.7</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="171">
@@ -6140,22 +6140,22 @@
       </c>
       <c r="B171" s="2" t="inlineStr">
         <is>
-          <t>Fitness age</t>
+          <t>Metrics engine</t>
         </is>
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>src/metrics/fitness-profile.test.ts</t>
+          <t>src/metrics/engine.test.ts</t>
         </is>
       </c>
       <c r="D171" s="3" t="inlineStr">
         <is>
-          <t>metricProfile</t>
+          <t>HRV outlier rein-in</t>
         </is>
       </c>
       <c r="E171" s="3" t="inlineStr">
         <is>
-          <t>a higher-is-better metric trending down reads "bad"</t>
+          <t>resting heart rate can be read from your sleep instead of the daily figure</t>
         </is>
       </c>
       <c r="F171" s="4" t="inlineStr">
@@ -6164,7 +6164,7 @@
         </is>
       </c>
       <c r="G171" s="5" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="172">
@@ -6188,7 +6188,7 @@
       </c>
       <c r="E172" s="3" t="inlineStr">
         <is>
-          <t>a lower-is-better metric (resting heart rate) flips the sign: a recent drop reads "good"</t>
+          <t>a higher-is-better metric trending up over the last 30 days reads "good"</t>
         </is>
       </c>
       <c r="F172" s="4" t="inlineStr">
@@ -6197,7 +6197,7 @@
         </is>
       </c>
       <c r="G172" s="5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="173">
@@ -6221,7 +6221,7 @@
       </c>
       <c r="E173" s="3" t="inlineStr">
         <is>
-          <t>years is capped and never wildly large</t>
+          <t>a higher-is-better metric trending down reads "bad"</t>
         </is>
       </c>
       <c r="F173" s="4" t="inlineStr">
@@ -6230,7 +6230,7 @@
         </is>
       </c>
       <c r="G173" s="5" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="174">
@@ -6254,7 +6254,7 @@
       </c>
       <c r="E174" s="3" t="inlineStr">
         <is>
-          <t>a flat metric reads "neutral"</t>
+          <t>a lower-is-better metric (resting heart rate) flips the sign: a recent drop reads "good"</t>
         </is>
       </c>
       <c r="F174" s="4" t="inlineStr">
@@ -6263,7 +6263,7 @@
         </is>
       </c>
       <c r="G174" s="5" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="175">
@@ -6287,7 +6287,7 @@
       </c>
       <c r="E175" s="3" t="inlineStr">
         <is>
-          <t>returns null when there is no data at all for the metric</t>
+          <t>years is capped and never wildly large</t>
         </is>
       </c>
       <c r="F175" s="4" t="inlineStr">
@@ -6296,7 +6296,7 @@
         </is>
       </c>
       <c r="G175" s="5" t="n">
-        <v>0.3</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="176">
@@ -6320,7 +6320,7 @@
       </c>
       <c r="E176" s="3" t="inlineStr">
         <is>
-          <t>sums HR zones 2–3 (excluding the rest-dominated zone 1) and 4–5 separately from the day's zone minutes</t>
+          <t>a flat metric reads "neutral"</t>
         </is>
       </c>
       <c r="F176" s="4" t="inlineStr">
@@ -6329,7 +6329,7 @@
         </is>
       </c>
       <c r="G176" s="5" t="n">
-        <v>13.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="177">
@@ -6353,7 +6353,7 @@
       </c>
       <c r="E177" s="3" t="inlineStr">
         <is>
-          <t>sums strength-type workout minutes for the day, ignoring other workout types</t>
+          <t>returns null when there is no data at all for the metric</t>
         </is>
       </c>
       <c r="F177" s="4" t="inlineStr">
@@ -6362,7 +6362,7 @@
         </is>
       </c>
       <c r="G177" s="5" t="n">
-        <v>1.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="178">
@@ -6381,12 +6381,12 @@
       </c>
       <c r="D178" s="3" t="inlineStr">
         <is>
-          <t>fitnessTrend</t>
+          <t>metricProfile</t>
         </is>
       </c>
       <c r="E178" s="3" t="inlineStr">
         <is>
-          <t>returns null with fewer than two months of VO2 readings</t>
+          <t>sums HR zones 2–3 (excluding the rest-dominated zone 1) and 4–5 separately from the day's zone minutes</t>
         </is>
       </c>
       <c r="F178" s="4" t="inlineStr">
@@ -6395,7 +6395,7 @@
         </is>
       </c>
       <c r="G178" s="5" t="n">
-        <v>0.5</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="179">
@@ -6414,12 +6414,12 @@
       </c>
       <c r="D179" s="3" t="inlineStr">
         <is>
-          <t>fitnessTrend</t>
+          <t>metricProfile</t>
         </is>
       </c>
       <c r="E179" s="3" t="inlineStr">
         <is>
-          <t>improving when VO2 max has risen over recent months, declining when it has fallen</t>
+          <t>sums strength-type workout minutes for the day, ignoring other workout types</t>
         </is>
       </c>
       <c r="F179" s="4" t="inlineStr">
@@ -6428,7 +6428,7 @@
         </is>
       </c>
       <c r="G179" s="5" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="180">
@@ -6437,22 +6437,22 @@
       </c>
       <c r="B180" s="2" t="inlineStr">
         <is>
-          <t>Stress &amp; fitness age</t>
+          <t>Fitness age</t>
         </is>
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>src/metrics/stress-fitness.test.ts</t>
+          <t>src/metrics/fitness-profile.test.ts</t>
         </is>
       </c>
       <c r="D180" s="3" t="inlineStr">
         <is>
-          <t>stress</t>
+          <t>fitnessTrend</t>
         </is>
       </c>
       <c r="E180" s="3" t="inlineStr">
         <is>
-          <t>a normal day sits in the Low band; a day with high daytime HR is higher</t>
+          <t>returns null with fewer than two months of VO2 readings</t>
         </is>
       </c>
       <c r="F180" s="4" t="inlineStr">
@@ -6461,7 +6461,7 @@
         </is>
       </c>
       <c r="G180" s="5" t="n">
-        <v>5.1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="181">
@@ -6470,22 +6470,22 @@
       </c>
       <c r="B181" s="2" t="inlineStr">
         <is>
-          <t>Stress &amp; fitness age</t>
+          <t>Fitness age</t>
         </is>
       </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>src/metrics/stress-fitness.test.ts</t>
+          <t>src/metrics/fitness-profile.test.ts</t>
         </is>
       </c>
       <c r="D181" s="3" t="inlineStr">
         <is>
-          <t>stress</t>
+          <t>fitnessTrend</t>
         </is>
       </c>
       <c r="E181" s="3" t="inlineStr">
         <is>
-          <t>leaves out sleeping and moving hours</t>
+          <t>improving when VO2 max has risen over recent months, declining when it has fallen</t>
         </is>
       </c>
       <c r="F181" s="4" t="inlineStr">
@@ -6494,7 +6494,7 @@
         </is>
       </c>
       <c r="G181" s="5" t="n">
-        <v>1</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="182">
@@ -6518,7 +6518,7 @@
       </c>
       <c r="E182" s="3" t="inlineStr">
         <is>
-          <t>needs a baseline first and stays within 0–3</t>
+          <t>a normal day sits in the Low band; a day with high daytime HR is higher</t>
         </is>
       </c>
       <c r="F182" s="4" t="inlineStr">
@@ -6527,7 +6527,7 @@
         </is>
       </c>
       <c r="G182" s="5" t="n">
-        <v>1.7</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="183">
@@ -6551,7 +6551,7 @@
       </c>
       <c r="E183" s="3" t="inlineStr">
         <is>
-          <t>labels</t>
+          <t>leaves out sleeping and moving hours</t>
         </is>
       </c>
       <c r="F183" s="4" t="inlineStr">
@@ -6560,7 +6560,7 @@
         </is>
       </c>
       <c r="G183" s="5" t="n">
-        <v>0.3</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="184">
@@ -6579,12 +6579,12 @@
       </c>
       <c r="D184" s="3" t="inlineStr">
         <is>
-          <t>fitness age</t>
+          <t>stress</t>
         </is>
       </c>
       <c r="E184" s="3" t="inlineStr">
         <is>
-          <t>matches your real age when your VO2 max equals the median for that age</t>
+          <t>needs a baseline first and stays within 0–3</t>
         </is>
       </c>
       <c r="F184" s="4" t="inlineStr">
@@ -6593,7 +6593,7 @@
         </is>
       </c>
       <c r="G184" s="5" t="n">
-        <v>0.4</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="185">
@@ -6612,12 +6612,12 @@
       </c>
       <c r="D185" s="3" t="inlineStr">
         <is>
-          <t>fitness age</t>
+          <t>stress</t>
         </is>
       </c>
       <c r="E185" s="3" t="inlineStr">
         <is>
-          <t>is younger for higher VO2 max, older for lower, and clamped</t>
+          <t>labels</t>
         </is>
       </c>
       <c r="F185" s="4" t="inlineStr">
@@ -6626,7 +6626,7 @@
         </is>
       </c>
       <c r="G185" s="5" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="186">
@@ -6650,7 +6650,7 @@
       </c>
       <c r="E186" s="3" t="inlineStr">
         <is>
-          <t>uses sex-specific references</t>
+          <t>matches your real age when your VO2 max equals the median for that age</t>
         </is>
       </c>
       <c r="F186" s="4" t="inlineStr">
@@ -6659,7 +6659,7 @@
         </is>
       </c>
       <c r="G186" s="5" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="187">
@@ -6683,7 +6683,7 @@
       </c>
       <c r="E187" s="3" t="inlineStr">
         <is>
-          <t>summarises readings: smooths with the last 3, compares with real age, builds a monthly series</t>
+          <t>is younger for higher VO2 max, older for lower, and clamped</t>
         </is>
       </c>
       <c r="F187" s="4" t="inlineStr">
@@ -6692,7 +6692,7 @@
         </is>
       </c>
       <c r="G187" s="5" t="n">
-        <v>1.9</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="188">
@@ -6716,7 +6716,7 @@
       </c>
       <c r="E188" s="3" t="inlineStr">
         <is>
-          <t>returns null without readings</t>
+          <t>uses sex-specific references</t>
         </is>
       </c>
       <c r="F188" s="4" t="inlineStr">
@@ -6725,7 +6725,7 @@
         </is>
       </c>
       <c r="G188" s="5" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="189">
@@ -6749,7 +6749,7 @@
       </c>
       <c r="E189" s="3" t="inlineStr">
         <is>
-          <t>categories</t>
+          <t>summarises readings: smooths with the last 3, compares with real age, builds a monthly series</t>
         </is>
       </c>
       <c r="F189" s="4" t="inlineStr">
@@ -6758,7 +6758,7 @@
         </is>
       </c>
       <c r="G189" s="5" t="n">
-        <v>0.3</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="190">
@@ -6782,7 +6782,7 @@
       </c>
       <c r="E190" s="3" t="inlineStr">
         <is>
-          <t>bands "about the same" within a 9-month tolerance either side of real age, not just exact equality</t>
+          <t>returns null without readings</t>
         </is>
       </c>
       <c r="F190" s="4" t="inlineStr">
@@ -6791,7 +6791,7 @@
         </is>
       </c>
       <c r="G190" s="5" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="191">
@@ -6800,22 +6800,22 @@
       </c>
       <c r="B191" s="2" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Stress &amp; fitness age</t>
         </is>
       </c>
       <c r="C191" s="2" t="inlineStr">
         <is>
-          <t>src/notifications/notifications.test.ts</t>
+          <t>src/metrics/stress-fitness.test.ts</t>
         </is>
       </c>
       <c r="D191" s="3" t="inlineStr">
         <is>
-          <t>day model</t>
+          <t>fitness age</t>
         </is>
       </c>
       <c r="E191" s="3" t="inlineStr">
         <is>
-          <t>anchors the windows on the usual wake time, in a sensible order</t>
+          <t>categories</t>
         </is>
       </c>
       <c r="F191" s="4" t="inlineStr">
@@ -6824,7 +6824,7 @@
         </is>
       </c>
       <c r="G191" s="5" t="n">
-        <v>2.5</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="192">
@@ -6833,22 +6833,22 @@
       </c>
       <c r="B192" s="2" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Stress &amp; fitness age</t>
         </is>
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>src/notifications/notifications.test.ts</t>
+          <t>src/metrics/stress-fitness.test.ts</t>
         </is>
       </c>
       <c r="D192" s="3" t="inlineStr">
         <is>
-          <t>day model</t>
+          <t>fitness age</t>
         </is>
       </c>
       <c r="E192" s="3" t="inlineStr">
         <is>
-          <t>puts the caffeine cutoff 9 hours before bed</t>
+          <t>bands "about the same" within a 9-month tolerance either side of real age, not just exact equality</t>
         </is>
       </c>
       <c r="F192" s="4" t="inlineStr">
@@ -6857,7 +6857,7 @@
         </is>
       </c>
       <c r="G192" s="5" t="n">
-        <v>1.3</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="193">
@@ -6881,7 +6881,7 @@
       </c>
       <c r="E193" s="3" t="inlineStr">
         <is>
-          <t>a low-recovery day gets an earlier bedtime and a shorter focus window; an adjust-off day does not</t>
+          <t>anchors the windows on the usual wake time, in a sensible order</t>
         </is>
       </c>
       <c r="F193" s="4" t="inlineStr">
@@ -6890,7 +6890,7 @@
         </is>
       </c>
       <c r="G193" s="5" t="n">
-        <v>2.4</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="194">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="E194" s="3" t="inlineStr">
         <is>
-          <t>uses your own workout habit for the activity window once there are enough workouts</t>
+          <t>puts the caffeine cutoff 9 hours before bed</t>
         </is>
       </c>
       <c r="F194" s="4" t="inlineStr">
@@ -6923,7 +6923,7 @@
         </is>
       </c>
       <c r="G194" s="5" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="195">
@@ -6947,7 +6947,7 @@
       </c>
       <c r="E195" s="3" t="inlineStr">
         <is>
-          <t>falls back to a 07:00 wake and 23:00 bedtime when there are no nights yet</t>
+          <t>a low-recovery day gets an earlier bedtime and a shorter focus window; an adjust-off day does not</t>
         </is>
       </c>
       <c r="F195" s="4" t="inlineStr">
@@ -6956,7 +6956,7 @@
         </is>
       </c>
       <c r="G195" s="5" t="n">
-        <v>0.5</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="196">
@@ -6975,12 +6975,12 @@
       </c>
       <c r="D196" s="3" t="inlineStr">
         <is>
-          <t>plan</t>
+          <t>day model</t>
         </is>
       </c>
       <c r="E196" s="3" t="inlineStr">
         <is>
-          <t>is sorted by time, has unique stable ids and stays under the iOS limit</t>
+          <t>uses your own workout habit for the activity window once there are enough workouts</t>
         </is>
       </c>
       <c r="F196" s="4" t="inlineStr">
@@ -6989,7 +6989,7 @@
         </is>
       </c>
       <c r="G196" s="5" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="197">
@@ -7008,12 +7008,12 @@
       </c>
       <c r="D197" s="3" t="inlineStr">
         <is>
-          <t>plan</t>
+          <t>day model</t>
         </is>
       </c>
       <c r="E197" s="3" t="inlineStr">
         <is>
-          <t>keeps at least 20 minutes between two notifications</t>
+          <t>falls back to a 07:00 wake and 23:00 bedtime when there are no nights yet</t>
         </is>
       </c>
       <c r="F197" s="4" t="inlineStr">
@@ -7022,7 +7022,7 @@
         </is>
       </c>
       <c r="G197" s="5" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="198">
@@ -7046,7 +7046,7 @@
       </c>
       <c r="E198" s="3" t="inlineStr">
         <is>
-          <t>stays quiet while you should be asleep, except the bedtime reminder itself</t>
+          <t>is sorted by time, has unique stable ids and stays under the iOS limit</t>
         </is>
       </c>
       <c r="F198" s="4" t="inlineStr">
@@ -7055,7 +7055,7 @@
         </is>
       </c>
       <c r="G198" s="5" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="199">
@@ -7079,7 +7079,7 @@
       </c>
       <c r="E199" s="3" t="inlineStr">
         <is>
-          <t>custom quiet hours are respected</t>
+          <t>keeps at least 20 minutes between two notifications</t>
         </is>
       </c>
       <c r="F199" s="4" t="inlineStr">
@@ -7088,7 +7088,7 @@
         </is>
       </c>
       <c r="G199" s="5" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="200">
@@ -7112,7 +7112,7 @@
       </c>
       <c r="E200" s="3" t="inlineStr">
         <is>
-          <t>never sends more than the daily cap in a day and keeps the highest priorities</t>
+          <t>stays quiet while you should be asleep, except the bedtime reminder itself</t>
         </is>
       </c>
       <c r="F200" s="4" t="inlineStr">
@@ -7121,7 +7121,7 @@
         </is>
       </c>
       <c r="G200" s="5" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="201">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="E201" s="3" t="inlineStr">
         <is>
-          <t>a category that is switched off produces nothing</t>
+          <t>custom quiet hours are respected</t>
         </is>
       </c>
       <c r="F201" s="4" t="inlineStr">
@@ -7154,7 +7154,7 @@
         </is>
       </c>
       <c r="G201" s="5" t="n">
-        <v>1.4</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="202">
@@ -7178,7 +7178,7 @@
       </c>
       <c r="E202" s="3" t="inlineStr">
         <is>
-          <t>the hydration count is honoured (at most that many per day)</t>
+          <t>never sends more than the daily cap in a day and keeps the highest priorities</t>
         </is>
       </c>
       <c r="F202" s="4" t="inlineStr">
@@ -7187,7 +7187,7 @@
         </is>
       </c>
       <c r="G202" s="5" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="203">
@@ -7211,7 +7211,7 @@
       </c>
       <c r="E203" s="3" t="inlineStr">
         <is>
-          <t>the wind-down reminder comes exactly the chosen number of minutes before bed</t>
+          <t>a category that is switched off produces nothing</t>
         </is>
       </c>
       <c r="F203" s="4" t="inlineStr">
@@ -7220,7 +7220,7 @@
         </is>
       </c>
       <c r="G203" s="5" t="n">
-        <v>1.9</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="204">
@@ -7244,7 +7244,7 @@
       </c>
       <c r="E204" s="3" t="inlineStr">
         <is>
-          <t>uses the "early night" wording on a low-recovery day, the plain wind-down otherwise</t>
+          <t>the hydration count is honoured (at most that many per day)</t>
         </is>
       </c>
       <c r="F204" s="4" t="inlineStr">
@@ -7253,7 +7253,7 @@
         </is>
       </c>
       <c r="G204" s="5" t="n">
-        <v>1.7</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="205">
@@ -7277,7 +7277,7 @@
       </c>
       <c r="E205" s="3" t="inlineStr">
         <is>
-          <t>upcoming() drops what has passed</t>
+          <t>the wind-down reminder comes exactly the chosen number of minutes before bed</t>
         </is>
       </c>
       <c r="F205" s="4" t="inlineStr">
@@ -7286,7 +7286,7 @@
         </is>
       </c>
       <c r="G205" s="5" t="n">
-        <v>0.3</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="206">
@@ -7310,7 +7310,7 @@
       </c>
       <c r="E206" s="3" t="inlineStr">
         <is>
-          <t>counts what came due since the inbox was last opened, for today only</t>
+          <t>uses the "early night" wording on a low-recovery day, the plain wind-down otherwise</t>
         </is>
       </c>
       <c r="F206" s="4" t="inlineStr">
@@ -7319,7 +7319,7 @@
         </is>
       </c>
       <c r="G206" s="5" t="n">
-        <v>0.2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="207">
@@ -7343,7 +7343,7 @@
       </c>
       <c r="E207" s="3" t="inlineStr">
         <is>
-          <t>time helpers cross midnight correctly</t>
+          <t>upcoming() drops what has passed</t>
         </is>
       </c>
       <c r="F207" s="4" t="inlineStr">
@@ -7352,7 +7352,7 @@
         </is>
       </c>
       <c r="G207" s="5" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="208">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E208" s="3" t="inlineStr">
         <is>
-          <t>wording is friendly, never names another product and makes no medical claims</t>
+          <t>counts what came due since the inbox was last opened, for today only</t>
         </is>
       </c>
       <c r="F208" s="4" t="inlineStr">
@@ -7385,7 +7385,7 @@
         </is>
       </c>
       <c r="G208" s="5" t="n">
-        <v>1.6</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="209">
@@ -7394,22 +7394,22 @@
       </c>
       <c r="B209" s="2" t="inlineStr">
         <is>
-          <t>Home layout</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C209" s="2" t="inlineStr">
         <is>
-          <t>src/state/home-layout.test.ts</t>
+          <t>src/notifications/notifications.test.ts</t>
         </is>
       </c>
       <c r="D209" s="3" t="inlineStr">
         <is>
-          <t>normalizeLayout</t>
+          <t>plan</t>
         </is>
       </c>
       <c r="E209" s="3" t="inlineStr">
         <is>
-          <t>keeps a valid saved layout</t>
+          <t>time helpers cross midnight correctly</t>
         </is>
       </c>
       <c r="F209" s="4" t="inlineStr">
@@ -7418,7 +7418,7 @@
         </is>
       </c>
       <c r="G209" s="5" t="n">
-        <v>2.3</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="210">
@@ -7427,22 +7427,22 @@
       </c>
       <c r="B210" s="2" t="inlineStr">
         <is>
-          <t>Home layout</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C210" s="2" t="inlineStr">
         <is>
-          <t>src/state/home-layout.test.ts</t>
+          <t>src/notifications/notifications.test.ts</t>
         </is>
       </c>
       <c r="D210" s="3" t="inlineStr">
         <is>
-          <t>normalizeLayout</t>
+          <t>plan</t>
         </is>
       </c>
       <c r="E210" s="3" t="inlineStr">
         <is>
-          <t>always returns every widget exactly once, whatever was saved</t>
+          <t>wording is friendly, never names another product and makes no medical claims</t>
         </is>
       </c>
       <c r="F210" s="4" t="inlineStr">
@@ -7451,7 +7451,7 @@
         </is>
       </c>
       <c r="G210" s="5" t="n">
-        <v>0.7</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="211">
@@ -7475,7 +7475,7 @@
       </c>
       <c r="E211" s="3" t="inlineStr">
         <is>
-          <t>appends widgets added since the layout was saved, keeping the saved order first</t>
+          <t>keeps a valid saved layout</t>
         </is>
       </c>
       <c r="F211" s="4" t="inlineStr">
@@ -7484,7 +7484,7 @@
         </is>
       </c>
       <c r="G211" s="5" t="n">
-        <v>0.3</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="212">
@@ -7508,7 +7508,7 @@
       </c>
       <c r="E212" s="3" t="inlineStr">
         <is>
-          <t>drops unknown or duplicated hidden ids</t>
+          <t>always returns every widget exactly once, whatever was saved</t>
         </is>
       </c>
       <c r="F212" s="4" t="inlineStr">
@@ -7517,7 +7517,7 @@
         </is>
       </c>
       <c r="G212" s="5" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="213">
@@ -7541,7 +7541,7 @@
       </c>
       <c r="E213" s="3" t="inlineStr">
         <is>
-          <t>never lets the fixed date strip or score rings into the layout</t>
+          <t>appends widgets added since the layout was saved, keeping the saved order first</t>
         </is>
       </c>
       <c r="F213" s="4" t="inlineStr">
@@ -7550,7 +7550,7 @@
         </is>
       </c>
       <c r="G213" s="5" t="n">
-        <v>1.4</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="214">
@@ -7569,12 +7569,12 @@
       </c>
       <c r="D214" s="3" t="inlineStr">
         <is>
-          <t>visibleWidgets</t>
+          <t>normalizeLayout</t>
         </is>
       </c>
       <c r="E214" s="3" t="inlineStr">
         <is>
-          <t>leaves out anything hidden, keeping order</t>
+          <t>drops unknown or duplicated hidden ids</t>
         </is>
       </c>
       <c r="F214" s="4" t="inlineStr">
@@ -7583,7 +7583,7 @@
         </is>
       </c>
       <c r="G214" s="5" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="215">
@@ -7602,12 +7602,12 @@
       </c>
       <c r="D215" s="3" t="inlineStr">
         <is>
-          <t>visibleWidgets</t>
+          <t>normalizeLayout</t>
         </is>
       </c>
       <c r="E215" s="3" t="inlineStr">
         <is>
-          <t>can be empty when everything is hidden</t>
+          <t>never lets the fixed date strip or score rings into the layout</t>
         </is>
       </c>
       <c r="F215" s="4" t="inlineStr">
@@ -7616,7 +7616,7 @@
         </is>
       </c>
       <c r="G215" s="5" t="n">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="216">
@@ -7635,12 +7635,12 @@
       </c>
       <c r="D216" s="3" t="inlineStr">
         <is>
-          <t>packRows</t>
+          <t>visibleWidgets</t>
         </is>
       </c>
       <c r="E216" s="3" t="inlineStr">
         <is>
-          <t>pairs the two half-width tiles into one row, full-width widgets take their own</t>
+          <t>leaves out anything hidden, keeping order</t>
         </is>
       </c>
       <c r="F216" s="4" t="inlineStr">
@@ -7649,7 +7649,7 @@
         </is>
       </c>
       <c r="G216" s="5" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="217">
@@ -7668,12 +7668,12 @@
       </c>
       <c r="D217" s="3" t="inlineStr">
         <is>
-          <t>packRows</t>
+          <t>visibleWidgets</t>
         </is>
       </c>
       <c r="E217" s="3" t="inlineStr">
         <is>
-          <t>leaves a half-width tile alone in its row when its partner is hidden</t>
+          <t>can be empty when everything is hidden</t>
         </is>
       </c>
       <c r="F217" s="4" t="inlineStr">
@@ -7682,7 +7682,7 @@
         </is>
       </c>
       <c r="G217" s="5" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="218">
@@ -7706,7 +7706,7 @@
       </c>
       <c r="E218" s="3" t="inlineStr">
         <is>
-          <t>does not pair half-width tiles that are not next to each other</t>
+          <t>pairs the two half-width tiles into one row, full-width widgets take their own</t>
         </is>
       </c>
       <c r="F218" s="4" t="inlineStr">
@@ -7715,7 +7715,7 @@
         </is>
       </c>
       <c r="G218" s="5" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="219">
@@ -7739,7 +7739,7 @@
       </c>
       <c r="E219" s="3" t="inlineStr">
         <is>
-          <t>pairs them in whichever order the user put them</t>
+          <t>leaves a half-width tile alone in its row when its partner is hidden</t>
         </is>
       </c>
       <c r="F219" s="4" t="inlineStr">
@@ -7772,7 +7772,7 @@
       </c>
       <c r="E220" s="3" t="inlineStr">
         <is>
-          <t>never drops or duplicates a widget, and never puts more than two in a row</t>
+          <t>does not pair half-width tiles that are not next to each other</t>
         </is>
       </c>
       <c r="F220" s="4" t="inlineStr">
@@ -7781,7 +7781,7 @@
         </is>
       </c>
       <c r="G220" s="5" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="221">
@@ -7805,7 +7805,7 @@
       </c>
       <c r="E221" s="3" t="inlineStr">
         <is>
-          <t>knows which widgets are half-width</t>
+          <t>pairs them in whichever order the user put them</t>
         </is>
       </c>
       <c r="F221" s="4" t="inlineStr">
@@ -7814,7 +7814,7 @@
         </is>
       </c>
       <c r="G221" s="5" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="222">
@@ -7833,12 +7833,12 @@
       </c>
       <c r="D222" s="3" t="inlineStr">
         <is>
-          <t>moved</t>
+          <t>packRows</t>
         </is>
       </c>
       <c r="E222" s="3" t="inlineStr">
         <is>
-          <t>moves an item down and up, keeping every other item</t>
+          <t>never drops or duplicates a widget, and never puts more than two in a row</t>
         </is>
       </c>
       <c r="F222" s="4" t="inlineStr">
@@ -7866,12 +7866,12 @@
       </c>
       <c r="D223" s="3" t="inlineStr">
         <is>
-          <t>moved</t>
+          <t>packRows</t>
         </is>
       </c>
       <c r="E223" s="3" t="inlineStr">
         <is>
-          <t>is a no-op for the same or an out-of-range index</t>
+          <t>knows which widgets are half-width</t>
         </is>
       </c>
       <c r="F223" s="4" t="inlineStr">
@@ -7904,7 +7904,7 @@
       </c>
       <c r="E224" s="3" t="inlineStr">
         <is>
-          <t>never loses or duplicates an item</t>
+          <t>moves an item down and up, keeping every other item</t>
         </is>
       </c>
       <c r="F224" s="4" t="inlineStr">
@@ -7922,22 +7922,22 @@
       </c>
       <c r="B225" s="2" t="inlineStr">
         <is>
-          <t>intake-log</t>
+          <t>Home layout</t>
         </is>
       </c>
       <c r="C225" s="2" t="inlineStr">
         <is>
-          <t>src/state/intake-log.test.ts</t>
+          <t>src/state/home-layout.test.ts</t>
         </is>
       </c>
       <c r="D225" s="3" t="inlineStr">
         <is>
-          <t>dailyWaterMl</t>
+          <t>moved</t>
         </is>
       </c>
       <c r="E225" s="3" t="inlineStr">
         <is>
-          <t>returns one total per day, oldest first, ending today</t>
+          <t>is a no-op for the same or an out-of-range index</t>
         </is>
       </c>
       <c r="F225" s="4" t="inlineStr">
@@ -7946,7 +7946,7 @@
         </is>
       </c>
       <c r="G225" s="5" t="n">
-        <v>3.4</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="226">
@@ -7955,22 +7955,22 @@
       </c>
       <c r="B226" s="2" t="inlineStr">
         <is>
-          <t>intake-log</t>
+          <t>Home layout</t>
         </is>
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>src/state/intake-log.test.ts</t>
+          <t>src/state/home-layout.test.ts</t>
         </is>
       </c>
       <c r="D226" s="3" t="inlineStr">
         <is>
-          <t>dailyWaterMl</t>
+          <t>moved</t>
         </is>
       </c>
       <c r="E226" s="3" t="inlineStr">
         <is>
-          <t>sums each day’s water in ml, ignoring caffeine and other days</t>
+          <t>never loses or duplicates an item</t>
         </is>
       </c>
       <c r="F226" s="4" t="inlineStr">
@@ -7979,7 +7979,7 @@
         </is>
       </c>
       <c r="G226" s="5" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="227">
@@ -8003,7 +8003,7 @@
       </c>
       <c r="E227" s="3" t="inlineStr">
         <is>
-          <t>counts old entries without a size as one 250 ml glass</t>
+          <t>returns one total per day, oldest first, ending today</t>
         </is>
       </c>
       <c r="F227" s="4" t="inlineStr">
@@ -8012,7 +8012,7 @@
         </is>
       </c>
       <c r="G227" s="5" t="n">
-        <v>0.2</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="228">
@@ -8021,22 +8021,22 @@
       </c>
       <c r="B228" s="2" t="inlineStr">
         <is>
-          <t>Home rings</t>
+          <t>intake-log</t>
         </is>
       </c>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t>src/state/ring-order.test.ts</t>
+          <t>src/state/intake-log.test.ts</t>
         </is>
       </c>
       <c r="D228" s="3" t="inlineStr">
         <is>
-          <t>normalizeOrder</t>
+          <t>dailyWaterMl</t>
         </is>
       </c>
       <c r="E228" s="3" t="inlineStr">
         <is>
-          <t>keeps a valid saved order as-is</t>
+          <t>sums each day’s water in ml, ignoring caffeine and other days</t>
         </is>
       </c>
       <c r="F228" s="4" t="inlineStr">
@@ -8045,7 +8045,7 @@
         </is>
       </c>
       <c r="G228" s="5" t="n">
-        <v>1.6</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="229">
@@ -8054,22 +8054,22 @@
       </c>
       <c r="B229" s="2" t="inlineStr">
         <is>
-          <t>Home rings</t>
+          <t>intake-log</t>
         </is>
       </c>
       <c r="C229" s="2" t="inlineStr">
         <is>
-          <t>src/state/ring-order.test.ts</t>
+          <t>src/state/intake-log.test.ts</t>
         </is>
       </c>
       <c r="D229" s="3" t="inlineStr">
         <is>
-          <t>normalizeOrder</t>
+          <t>dailyWaterMl</t>
         </is>
       </c>
       <c r="E229" s="3" t="inlineStr">
         <is>
-          <t>falls back to the default for junk, and always returns all three rings</t>
+          <t>counts old entries without a size as one 250 ml glass</t>
         </is>
       </c>
       <c r="F229" s="4" t="inlineStr">
@@ -8078,7 +8078,7 @@
         </is>
       </c>
       <c r="G229" s="5" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="230">
@@ -8102,7 +8102,7 @@
       </c>
       <c r="E230" s="3" t="inlineStr">
         <is>
-          <t>appends anything missing, keeping the saved part first</t>
+          <t>keeps a valid saved order as-is</t>
         </is>
       </c>
       <c r="F230" s="4" t="inlineStr">
@@ -8111,7 +8111,7 @@
         </is>
       </c>
       <c r="G230" s="5" t="n">
-        <v>0.2</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="231">
@@ -8130,12 +8130,12 @@
       </c>
       <c r="D231" s="3" t="inlineStr">
         <is>
-          <t>swapped</t>
+          <t>normalizeOrder</t>
         </is>
       </c>
       <c r="E231" s="3" t="inlineStr">
         <is>
-          <t>swaps the two rings and stays a permutation</t>
+          <t>falls back to the default for junk, and always returns all three rings</t>
         </is>
       </c>
       <c r="F231" s="4" t="inlineStr">
@@ -8144,7 +8144,7 @@
         </is>
       </c>
       <c r="G231" s="5" t="n">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="232">
@@ -8163,12 +8163,12 @@
       </c>
       <c r="D232" s="3" t="inlineStr">
         <is>
-          <t>swapped</t>
+          <t>normalizeOrder</t>
         </is>
       </c>
       <c r="E232" s="3" t="inlineStr">
         <is>
-          <t>is a no-op when the ring is already in that position</t>
+          <t>appends anything missing, keeping the saved part first</t>
         </is>
       </c>
       <c r="F232" s="4" t="inlineStr">
@@ -8177,7 +8177,7 @@
         </is>
       </c>
       <c r="G232" s="5" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="233">
@@ -8201,7 +8201,7 @@
       </c>
       <c r="E233" s="3" t="inlineStr">
         <is>
-          <t>ignores an out-of-range position</t>
+          <t>swaps the two rings and stays a permutation</t>
         </is>
       </c>
       <c r="F233" s="4" t="inlineStr">
@@ -8234,20 +8234,86 @@
       </c>
       <c r="E234" s="3" t="inlineStr">
         <is>
+          <t>is a no-op when the ring is already in that position</t>
+        </is>
+      </c>
+      <c r="F234" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G234" s="5" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="2" t="n">
+        <v>234</v>
+      </c>
+      <c r="B235" s="2" t="inlineStr">
+        <is>
+          <t>Home rings</t>
+        </is>
+      </c>
+      <c r="C235" s="2" t="inlineStr">
+        <is>
+          <t>src/state/ring-order.test.ts</t>
+        </is>
+      </c>
+      <c r="D235" s="3" t="inlineStr">
+        <is>
+          <t>swapped</t>
+        </is>
+      </c>
+      <c r="E235" s="3" t="inlineStr">
+        <is>
+          <t>ignores an out-of-range position</t>
+        </is>
+      </c>
+      <c r="F235" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G235" s="5" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="2" t="n">
+        <v>235</v>
+      </c>
+      <c r="B236" s="2" t="inlineStr">
+        <is>
+          <t>Home rings</t>
+        </is>
+      </c>
+      <c r="C236" s="2" t="inlineStr">
+        <is>
+          <t>src/state/ring-order.test.ts</t>
+        </is>
+      </c>
+      <c r="D236" s="3" t="inlineStr">
+        <is>
+          <t>swapped</t>
+        </is>
+      </c>
+      <c r="E236" s="3" t="inlineStr">
+        <is>
           <t>any sequence of swaps leaves every ring present exactly once</t>
         </is>
       </c>
-      <c r="F234" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G234" s="5" t="n">
-        <v>0.3</v>
+      <c r="F236" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G236" s="5" t="n">
+        <v>0.2</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G234"/>
+  <autoFilter ref="A1:G236"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8275,7 +8341,7 @@
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>Generated 2026-10-04 12:08 UTC from a live vitest run</t>
+          <t>Generated 2026-10-04 13:00 UTC from a live vitest run</t>
         </is>
       </c>
     </row>
@@ -8293,7 +8359,7 @@
         </is>
       </c>
       <c r="B5" s="10">
-        <f>COUNTA('Test Cases'!$A$2:$A$234)</f>
+        <f>COUNTA('Test Cases'!$A$2:$A$236)</f>
         <v/>
       </c>
     </row>
@@ -8304,7 +8370,7 @@
         </is>
       </c>
       <c r="B6" s="10">
-        <f>COUNTIF('Test Cases'!$F$2:$F$234,"passed")</f>
+        <f>COUNTIF('Test Cases'!$F$2:$F$236,"passed")</f>
         <v/>
       </c>
     </row>
@@ -8315,7 +8381,7 @@
         </is>
       </c>
       <c r="B7" s="11">
-        <f>COUNTA('Test Cases'!$A$2:$A$234)-COUNTIF('Test Cases'!$F$2:$F$234,"passed")</f>
+        <f>COUNTA('Test Cases'!$A$2:$A$236)-COUNTIF('Test Cases'!$F$2:$F$236,"passed")</f>
         <v/>
       </c>
     </row>
@@ -8357,7 +8423,7 @@
         </is>
       </c>
       <c r="B12" s="14">
-        <f>COUNTIF('Test Cases'!$B$2:$B$234,$A12)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$236,$A12)</f>
         <v/>
       </c>
     </row>
@@ -8368,7 +8434,7 @@
         </is>
       </c>
       <c r="B13" s="14">
-        <f>COUNTIF('Test Cases'!$B$2:$B$234,$A13)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$236,$A13)</f>
         <v/>
       </c>
     </row>
@@ -8379,7 +8445,7 @@
         </is>
       </c>
       <c r="B14" s="14">
-        <f>COUNTIF('Test Cases'!$B$2:$B$234,$A14)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$236,$A14)</f>
         <v/>
       </c>
     </row>
@@ -8390,7 +8456,7 @@
         </is>
       </c>
       <c r="B15" s="14">
-        <f>COUNTIF('Test Cases'!$B$2:$B$234,$A15)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$236,$A15)</f>
         <v/>
       </c>
     </row>
@@ -8401,7 +8467,7 @@
         </is>
       </c>
       <c r="B16" s="14">
-        <f>COUNTIF('Test Cases'!$B$2:$B$234,$A16)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$236,$A16)</f>
         <v/>
       </c>
     </row>
@@ -8412,7 +8478,7 @@
         </is>
       </c>
       <c r="B17" s="14">
-        <f>COUNTIF('Test Cases'!$B$2:$B$234,$A17)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$236,$A17)</f>
         <v/>
       </c>
     </row>
@@ -8423,7 +8489,7 @@
         </is>
       </c>
       <c r="B18" s="14">
-        <f>COUNTIF('Test Cases'!$B$2:$B$234,$A18)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$236,$A18)</f>
         <v/>
       </c>
     </row>
@@ -8434,7 +8500,7 @@
         </is>
       </c>
       <c r="B19" s="14">
-        <f>COUNTIF('Test Cases'!$B$2:$B$234,$A19)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$236,$A19)</f>
         <v/>
       </c>
     </row>
@@ -8445,7 +8511,7 @@
         </is>
       </c>
       <c r="B20" s="14">
-        <f>COUNTIF('Test Cases'!$B$2:$B$234,$A20)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$236,$A20)</f>
         <v/>
       </c>
     </row>
@@ -8456,7 +8522,7 @@
         </is>
       </c>
       <c r="B21" s="14">
-        <f>COUNTIF('Test Cases'!$B$2:$B$234,$A21)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$236,$A21)</f>
         <v/>
       </c>
     </row>
@@ -8467,7 +8533,7 @@
         </is>
       </c>
       <c r="B22" s="14">
-        <f>COUNTIF('Test Cases'!$B$2:$B$234,$A22)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$236,$A22)</f>
         <v/>
       </c>
     </row>
@@ -8478,7 +8544,7 @@
         </is>
       </c>
       <c r="B23" s="14">
-        <f>COUNTIF('Test Cases'!$B$2:$B$234,$A23)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$236,$A23)</f>
         <v/>
       </c>
     </row>
@@ -8489,7 +8555,7 @@
         </is>
       </c>
       <c r="B24" s="14">
-        <f>COUNTIF('Test Cases'!$B$2:$B$234,$A24)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$236,$A24)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Import: keep four years of history before the export date (was two)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="G2" s="5" t="n">
-        <v>11.3</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="3">
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="G3" s="5" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="4">
@@ -851,7 +851,7 @@
         </is>
       </c>
       <c r="G10" s="5" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="11">
@@ -884,7 +884,7 @@
         </is>
       </c>
       <c r="G11" s="5" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="12">
@@ -917,7 +917,7 @@
         </is>
       </c>
       <c r="G12" s="5" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="13">
@@ -950,7 +950,7 @@
         </is>
       </c>
       <c r="G13" s="5" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="14">
@@ -1016,7 +1016,7 @@
         </is>
       </c>
       <c r="G15" s="5" t="n">
-        <v>2.7</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="16">
@@ -1049,7 +1049,7 @@
         </is>
       </c>
       <c r="G16" s="5" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="17">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="G17" s="5" t="n">
-        <v>1.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -1115,7 +1115,7 @@
         </is>
       </c>
       <c r="G18" s="5" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="19">
@@ -1148,7 +1148,7 @@
         </is>
       </c>
       <c r="G19" s="5" t="n">
-        <v>2.4</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="20">
@@ -1181,7 +1181,7 @@
         </is>
       </c>
       <c r="G20" s="5" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="21">
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="G21" s="5" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="22">
@@ -1247,7 +1247,7 @@
         </is>
       </c>
       <c r="G22" s="5" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="23">
@@ -1280,7 +1280,7 @@
         </is>
       </c>
       <c r="G23" s="5" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="24">
@@ -1379,7 +1379,7 @@
         </is>
       </c>
       <c r="G26" s="5" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="27">
@@ -1412,7 +1412,7 @@
         </is>
       </c>
       <c r="G27" s="5" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="28">
@@ -1511,7 +1511,7 @@
         </is>
       </c>
       <c r="G30" s="5" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="31">
@@ -1544,7 +1544,7 @@
         </is>
       </c>
       <c r="G31" s="5" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="32">
@@ -1775,7 +1775,7 @@
         </is>
       </c>
       <c r="G38" s="5" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="39">
@@ -1808,7 +1808,7 @@
         </is>
       </c>
       <c r="G39" s="5" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="40">
@@ -2468,7 +2468,7 @@
         </is>
       </c>
       <c r="G59" s="5" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="60">
@@ -2534,7 +2534,7 @@
         </is>
       </c>
       <c r="G61" s="5" t="n">
-        <v>0.1</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="62">
@@ -2567,7 +2567,7 @@
         </is>
       </c>
       <c r="G62" s="5" t="n">
-        <v>1.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="63">
@@ -3425,7 +3425,7 @@
         </is>
       </c>
       <c r="G88" s="5" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="89">
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="G91" s="5" t="n">
-        <v>2.3</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="92">
@@ -3557,7 +3557,7 @@
         </is>
       </c>
       <c r="G92" s="5" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="93">
@@ -3590,7 +3590,7 @@
         </is>
       </c>
       <c r="G93" s="5" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="94">
@@ -3623,7 +3623,7 @@
         </is>
       </c>
       <c r="G94" s="5" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="95">
@@ -3689,7 +3689,7 @@
         </is>
       </c>
       <c r="G96" s="5" t="n">
-        <v>3.5</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="97">
@@ -3755,7 +3755,7 @@
         </is>
       </c>
       <c r="G98" s="5" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="99">
@@ -3821,7 +3821,7 @@
         </is>
       </c>
       <c r="G100" s="5" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="101">
@@ -3854,7 +3854,7 @@
         </is>
       </c>
       <c r="G101" s="5" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="102">
@@ -3887,7 +3887,7 @@
         </is>
       </c>
       <c r="G102" s="5" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="103">
@@ -3920,7 +3920,7 @@
         </is>
       </c>
       <c r="G103" s="5" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="104">
@@ -3953,7 +3953,7 @@
         </is>
       </c>
       <c r="G104" s="5" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="105">
@@ -3986,7 +3986,7 @@
         </is>
       </c>
       <c r="G105" s="5" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="106">
@@ -4019,7 +4019,7 @@
         </is>
       </c>
       <c r="G106" s="5" t="n">
-        <v>12.4</v>
+        <v>12</v>
       </c>
     </row>
     <row r="107">
@@ -4052,7 +4052,7 @@
         </is>
       </c>
       <c r="G107" s="5" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="108">
@@ -4085,7 +4085,7 @@
         </is>
       </c>
       <c r="G108" s="5" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="109">
@@ -4118,7 +4118,7 @@
         </is>
       </c>
       <c r="G109" s="5" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="110">
@@ -4217,7 +4217,7 @@
         </is>
       </c>
       <c r="G112" s="5" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="113">
@@ -4316,7 +4316,7 @@
         </is>
       </c>
       <c r="G115" s="5" t="n">
-        <v>5.3</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="116">
@@ -4349,7 +4349,7 @@
         </is>
       </c>
       <c r="G116" s="5" t="n">
-        <v>24.5</v>
+        <v>18.9</v>
       </c>
     </row>
     <row r="117">
@@ -4382,7 +4382,7 @@
         </is>
       </c>
       <c r="G117" s="5" t="n">
-        <v>232.3</v>
+        <v>225.6</v>
       </c>
     </row>
     <row r="118">
@@ -4415,7 +4415,7 @@
         </is>
       </c>
       <c r="G118" s="5" t="n">
-        <v>15.6</v>
+        <v>15.7</v>
       </c>
     </row>
     <row r="119">
@@ -4448,7 +4448,7 @@
         </is>
       </c>
       <c r="G119" s="5" t="n">
-        <v>14.7</v>
+        <v>14.5</v>
       </c>
     </row>
     <row r="120">
@@ -4481,7 +4481,7 @@
         </is>
       </c>
       <c r="G120" s="5" t="n">
-        <v>1.9</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="121">
@@ -4514,7 +4514,7 @@
         </is>
       </c>
       <c r="G121" s="5" t="n">
-        <v>28.4</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="122">
@@ -4547,7 +4547,7 @@
         </is>
       </c>
       <c r="G122" s="5" t="n">
-        <v>15.6</v>
+        <v>15.9</v>
       </c>
     </row>
     <row r="123">
@@ -4580,7 +4580,7 @@
         </is>
       </c>
       <c r="G123" s="5" t="n">
-        <v>5.7</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="124">
@@ -4613,7 +4613,7 @@
         </is>
       </c>
       <c r="G124" s="5" t="n">
-        <v>1.2</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="125">
@@ -4646,7 +4646,7 @@
         </is>
       </c>
       <c r="G125" s="5" t="n">
-        <v>0.9</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="126">
@@ -4679,7 +4679,7 @@
         </is>
       </c>
       <c r="G126" s="5" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="127">
@@ -4712,7 +4712,7 @@
         </is>
       </c>
       <c r="G127" s="5" t="n">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="128">
@@ -4745,7 +4745,7 @@
         </is>
       </c>
       <c r="G128" s="5" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="129">
@@ -4769,7 +4769,7 @@
       </c>
       <c r="E129" s="3" t="inlineStr">
         <is>
-          <t>keeps the two years before the export date and ignores lines it does not know (header, DTD)</t>
+          <t>keeps the four years before the export date and ignores lines it does not know (header, DTD)</t>
         </is>
       </c>
       <c r="F129" s="4" t="inlineStr">
@@ -4778,7 +4778,7 @@
         </is>
       </c>
       <c r="G129" s="5" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="130">
@@ -4811,7 +4811,7 @@
         </is>
       </c>
       <c r="G130" s="5" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="131">
@@ -4835,7 +4835,7 @@
       </c>
       <c r="E131" s="3" t="inlineStr">
         <is>
-          <t>falls back to two years before today without an export date, and a fixed cutoff overrides both</t>
+          <t>falls back to four years before today without an export date, and a fixed cutoff overrides both</t>
         </is>
       </c>
       <c r="F131" s="4" t="inlineStr">
@@ -4844,7 +4844,7 @@
         </is>
       </c>
       <c r="G131" s="5" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="132">
@@ -4877,7 +4877,7 @@
         </is>
       </c>
       <c r="G132" s="5" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="133">
@@ -4910,7 +4910,7 @@
         </is>
       </c>
       <c r="G133" s="5" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="134">
@@ -4943,7 +4943,7 @@
         </is>
       </c>
       <c r="G134" s="5" t="n">
-        <v>6.9</v>
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="135">
@@ -5009,7 +5009,7 @@
         </is>
       </c>
       <c r="G136" s="5" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="137">
@@ -5075,7 +5075,7 @@
         </is>
       </c>
       <c r="G138" s="5" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="139">
@@ -5207,7 +5207,7 @@
         </is>
       </c>
       <c r="G142" s="5" t="n">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="143">
@@ -5240,7 +5240,7 @@
         </is>
       </c>
       <c r="G143" s="5" t="n">
-        <v>1.3</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="144">
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="G144" s="5" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="145">
@@ -5306,7 +5306,7 @@
         </is>
       </c>
       <c r="G145" s="5" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="146">
@@ -5339,7 +5339,7 @@
         </is>
       </c>
       <c r="G146" s="5" t="n">
-        <v>2.2</v>
+        <v>2</v>
       </c>
     </row>
     <row r="147">
@@ -5372,7 +5372,7 @@
         </is>
       </c>
       <c r="G147" s="5" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="148">
@@ -5405,7 +5405,7 @@
         </is>
       </c>
       <c r="G148" s="5" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="149">
@@ -5471,7 +5471,7 @@
         </is>
       </c>
       <c r="G150" s="5" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="151">
@@ -5504,7 +5504,7 @@
         </is>
       </c>
       <c r="G151" s="5" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="152">
@@ -5537,7 +5537,7 @@
         </is>
       </c>
       <c r="G152" s="5" t="n">
-        <v>2.3</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="153">
@@ -5570,7 +5570,7 @@
         </is>
       </c>
       <c r="G153" s="5" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="154">
@@ -5603,7 +5603,7 @@
         </is>
       </c>
       <c r="G154" s="5" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="155">
@@ -5669,7 +5669,7 @@
         </is>
       </c>
       <c r="G156" s="5" t="n">
-        <v>3</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="157">
@@ -5702,7 +5702,7 @@
         </is>
       </c>
       <c r="G157" s="5" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="158">
@@ -5735,7 +5735,7 @@
         </is>
       </c>
       <c r="G158" s="5" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="159">
@@ -5768,7 +5768,7 @@
         </is>
       </c>
       <c r="G159" s="5" t="n">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="160">
@@ -5801,7 +5801,7 @@
         </is>
       </c>
       <c r="G160" s="5" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="161">
@@ -5834,7 +5834,7 @@
         </is>
       </c>
       <c r="G161" s="5" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="162">
@@ -5867,7 +5867,7 @@
         </is>
       </c>
       <c r="G162" s="5" t="n">
-        <v>0.8</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="163">
@@ -5900,7 +5900,7 @@
         </is>
       </c>
       <c r="G163" s="5" t="n">
-        <v>1</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="164">
@@ -5933,7 +5933,7 @@
         </is>
       </c>
       <c r="G164" s="5" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="165">
@@ -5966,7 +5966,7 @@
         </is>
       </c>
       <c r="G165" s="5" t="n">
-        <v>1.1</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="166">
@@ -5999,7 +5999,7 @@
         </is>
       </c>
       <c r="G166" s="5" t="n">
-        <v>1</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="167">
@@ -6032,7 +6032,7 @@
         </is>
       </c>
       <c r="G167" s="5" t="n">
-        <v>1.7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="168">
@@ -6065,7 +6065,7 @@
         </is>
       </c>
       <c r="G168" s="5" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="169">
@@ -6098,7 +6098,7 @@
         </is>
       </c>
       <c r="G169" s="5" t="n">
-        <v>0.4</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="170">
@@ -6131,7 +6131,7 @@
         </is>
       </c>
       <c r="G170" s="5" t="n">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="171">
@@ -6164,7 +6164,7 @@
         </is>
       </c>
       <c r="G171" s="5" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="172">
@@ -6197,7 +6197,7 @@
         </is>
       </c>
       <c r="G172" s="5" t="n">
-        <v>4</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="173">
@@ -6230,7 +6230,7 @@
         </is>
       </c>
       <c r="G173" s="5" t="n">
-        <v>1.2</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="174">
@@ -6263,7 +6263,7 @@
         </is>
       </c>
       <c r="G174" s="5" t="n">
-        <v>1.1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="175">
@@ -6329,7 +6329,7 @@
         </is>
       </c>
       <c r="G176" s="5" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="177">
@@ -6395,7 +6395,7 @@
         </is>
       </c>
       <c r="G178" s="5" t="n">
-        <v>14.3</v>
+        <v>17.8</v>
       </c>
     </row>
     <row r="179">
@@ -6428,7 +6428,7 @@
         </is>
       </c>
       <c r="G179" s="5" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="180">
@@ -6494,7 +6494,7 @@
         </is>
       </c>
       <c r="G181" s="5" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="182">
@@ -6527,7 +6527,7 @@
         </is>
       </c>
       <c r="G182" s="5" t="n">
-        <v>5.4</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="183">
@@ -6560,7 +6560,7 @@
         </is>
       </c>
       <c r="G183" s="5" t="n">
-        <v>1.5</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="184">
@@ -6593,7 +6593,7 @@
         </is>
       </c>
       <c r="G184" s="5" t="n">
-        <v>2.2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="185">
@@ -6626,7 +6626,7 @@
         </is>
       </c>
       <c r="G185" s="5" t="n">
-        <v>0.2</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="186">
@@ -6659,7 +6659,7 @@
         </is>
       </c>
       <c r="G186" s="5" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="187">
@@ -6758,7 +6758,7 @@
         </is>
       </c>
       <c r="G189" s="5" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="190">
@@ -6890,7 +6890,7 @@
         </is>
       </c>
       <c r="G193" s="5" t="n">
-        <v>3.1</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="194">
@@ -6923,7 +6923,7 @@
         </is>
       </c>
       <c r="G194" s="5" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="195">
@@ -6956,7 +6956,7 @@
         </is>
       </c>
       <c r="G195" s="5" t="n">
-        <v>2.5</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="196">
@@ -6989,7 +6989,7 @@
         </is>
       </c>
       <c r="G196" s="5" t="n">
-        <v>1.4</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="197">
@@ -7022,7 +7022,7 @@
         </is>
       </c>
       <c r="G197" s="5" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="198">
@@ -7055,7 +7055,7 @@
         </is>
       </c>
       <c r="G198" s="5" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="199">
@@ -7088,7 +7088,7 @@
         </is>
       </c>
       <c r="G199" s="5" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="200">
@@ -7121,7 +7121,7 @@
         </is>
       </c>
       <c r="G200" s="5" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="201">
@@ -7154,7 +7154,7 @@
         </is>
       </c>
       <c r="G201" s="5" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="202">
@@ -7187,7 +7187,7 @@
         </is>
       </c>
       <c r="G202" s="5" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="203">
@@ -7220,7 +7220,7 @@
         </is>
       </c>
       <c r="G203" s="5" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="204">
@@ -7286,7 +7286,7 @@
         </is>
       </c>
       <c r="G205" s="5" t="n">
-        <v>2.5</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="206">
@@ -7319,7 +7319,7 @@
         </is>
       </c>
       <c r="G206" s="5" t="n">
-        <v>1.5</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="207">
@@ -7352,7 +7352,7 @@
         </is>
       </c>
       <c r="G207" s="5" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="208">
@@ -7451,7 +7451,7 @@
         </is>
       </c>
       <c r="G210" s="5" t="n">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="211">
@@ -7484,7 +7484,7 @@
         </is>
       </c>
       <c r="G211" s="5" t="n">
-        <v>2.6</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="212">
@@ -7517,7 +7517,7 @@
         </is>
       </c>
       <c r="G212" s="5" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="213">
@@ -7550,7 +7550,7 @@
         </is>
       </c>
       <c r="G213" s="5" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="214">
@@ -7583,7 +7583,7 @@
         </is>
       </c>
       <c r="G214" s="5" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="215">
@@ -7616,7 +7616,7 @@
         </is>
       </c>
       <c r="G215" s="5" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="216">
@@ -7682,7 +7682,7 @@
         </is>
       </c>
       <c r="G217" s="5" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="218">
@@ -7715,7 +7715,7 @@
         </is>
       </c>
       <c r="G218" s="5" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="219">
@@ -7847,7 +7847,7 @@
         </is>
       </c>
       <c r="G222" s="5" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="223">
@@ -7880,7 +7880,7 @@
         </is>
       </c>
       <c r="G223" s="5" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="224">
@@ -7913,7 +7913,7 @@
         </is>
       </c>
       <c r="G224" s="5" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="225">
@@ -7946,7 +7946,7 @@
         </is>
       </c>
       <c r="G225" s="5" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="226">
@@ -7979,7 +7979,7 @@
         </is>
       </c>
       <c r="G226" s="5" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="227">
@@ -8012,7 +8012,7 @@
         </is>
       </c>
       <c r="G227" s="5" t="n">
-        <v>2.8</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="228">
@@ -8045,7 +8045,7 @@
         </is>
       </c>
       <c r="G228" s="5" t="n">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="229">
@@ -8078,7 +8078,7 @@
         </is>
       </c>
       <c r="G229" s="5" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="230">
@@ -8111,7 +8111,7 @@
         </is>
       </c>
       <c r="G230" s="5" t="n">
-        <v>2.6</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="231">
@@ -8144,7 +8144,7 @@
         </is>
       </c>
       <c r="G231" s="5" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="232">
@@ -8177,7 +8177,7 @@
         </is>
       </c>
       <c r="G232" s="5" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="233">
@@ -8243,7 +8243,7 @@
         </is>
       </c>
       <c r="G234" s="5" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="235">
@@ -8276,7 +8276,7 @@
         </is>
       </c>
       <c r="G235" s="5" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="236">
@@ -8341,7 +8341,7 @@
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>Generated 2026-10-04 13:00 UTC from a live vitest run</t>
+          <t>Generated 2026-10-04 13:16 UTC from a live vitest run</t>
         </is>
       </c>
     </row>

</xml_diff>